<commit_message>
Cargar las luces de las losas y resolver las dos cruzadas
Diez losas en dos niveles. L02 y L08 se calculan como voladizo.
L07 (4,85x5,60) y L10 (4,85x6,00) apoyan en los cuatro bordes: se
reparte la carga por Marcus y ocupan un renglon por direccion.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planilla_losas.xlsx
+++ b/planillas/planilla_losas.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Planilla losas'!$1:$3</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Planilla losas'!$A$1:$R$13</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Planilla losas'!$A$1:$R$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -92,7 +92,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFE699"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -174,7 +174,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -220,7 +220,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -235,15 +235,21 @@
     <xf numFmtId="2" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="2" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="2" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -263,6 +269,12 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -601,6 +613,56 @@
     </pic>
     <clientData/>
   </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="11" name="Image 11" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId11"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="12" name="Image 12" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId12"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -1272,7 +1334,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R13"/>
+  <dimension ref="A1:T15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1292,7 +1354,9 @@
     <col width="8" customWidth="1" min="15" max="15"/>
     <col width="9" customWidth="1" min="16" max="16"/>
     <col width="9" customWidth="1" min="17" max="17"/>
-    <col width="34" customWidth="1" min="18" max="18"/>
+    <col width="40" customWidth="1" min="18" max="18"/>
+    <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="8" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -1365,6 +1429,12 @@
           <t>OBSERVACIONES</t>
         </is>
       </c>
+      <c r="S2" s="8" t="inlineStr">
+        <is>
+          <t>DATOS AUXILIARES</t>
+        </is>
+      </c>
+      <c r="T2" s="17" t="n"/>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="17" t="n"/>
@@ -1433,6 +1503,16 @@
         </is>
       </c>
       <c r="R3" s="17" t="n"/>
+      <c r="S3" s="18" t="inlineStr">
+        <is>
+          <t>luz transv.</t>
+        </is>
+      </c>
+      <c r="T3" s="18" t="inlineStr">
+        <is>
+          <t>k carga</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="46" customHeight="1">
       <c r="A4" s="19" t="inlineStr">
@@ -1445,14 +1525,16 @@
           <t>L01</t>
         </is>
       </c>
-      <c r="C4" s="21" t="n"/>
+      <c r="C4" s="21" t="n">
+        <v>3.65</v>
+      </c>
       <c r="D4" s="22" t="inlineStr">
         <is>
           <t>1/8</t>
         </is>
       </c>
       <c r="E4" s="23">
-        <f>Datos!$B$9*H4/100+VLOOKUP($A$4,Datos!$A$16:$C$17,2,0)+VLOOKUP($A$4,Datos!$A$16:$C$17,3,0)</f>
+        <f>(Datos!$B$9*H4/100+VLOOKUP($A$4,Datos!$A$16:$C$17,2,0)+VLOOKUP($A$4,Datos!$A$16:$C$17,3,0))*T4</f>
         <v/>
       </c>
       <c r="F4" s="7" t="n"/>
@@ -1497,27 +1579,30 @@
         <f>IF(C4="","",IF(VLOOKUP(D4,Datos!$A$21:$D$25,4,0)="Voladizo","---",P4))</f>
         <v/>
       </c>
-      <c r="R4" s="26" t="inlineStr">
-        <is>
-          <t>Falta la luz: completar en la columna LUZ y recalcula todo.</t>
-        </is>
+      <c r="R4" s="10" t="n"/>
+      <c r="S4" s="26" t="n"/>
+      <c r="T4" s="27">
+        <f>IF(S4="",1,S4^4/(C4^4+S4^4))</f>
+        <v/>
       </c>
     </row>
     <row r="5" ht="46" customHeight="1">
-      <c r="A5" s="27" t="n"/>
+      <c r="A5" s="28" t="n"/>
       <c r="B5" s="20" t="inlineStr">
         <is>
           <t>L02</t>
         </is>
       </c>
-      <c r="C5" s="21" t="n"/>
+      <c r="C5" s="21" t="n">
+        <v>0.8</v>
+      </c>
       <c r="D5" s="22" t="inlineStr">
         <is>
-          <t>1/8</t>
+          <t>1/2</t>
         </is>
       </c>
       <c r="E5" s="23">
-        <f>Datos!$B$9*H5/100+VLOOKUP($A$4,Datos!$A$16:$C$17,2,0)+VLOOKUP($A$4,Datos!$A$16:$C$17,3,0)</f>
+        <f>(Datos!$B$9*H5/100+VLOOKUP($A$4,Datos!$A$16:$C$17,2,0)+VLOOKUP($A$4,Datos!$A$16:$C$17,3,0))*T5</f>
         <v/>
       </c>
       <c r="F5" s="7" t="n"/>
@@ -1562,27 +1647,34 @@
         <f>IF(C5="","",IF(VLOOKUP(D5,Datos!$A$21:$D$25,4,0)="Voladizo","---",P5))</f>
         <v/>
       </c>
-      <c r="R5" s="26" t="inlineStr">
-        <is>
-          <t>Falta la luz: completar en la columna LUZ y recalcula todo.</t>
-        </is>
+      <c r="R5" s="29" t="inlineStr">
+        <is>
+          <t>Voladizo: un solo apoyo.</t>
+        </is>
+      </c>
+      <c r="S5" s="26" t="n"/>
+      <c r="T5" s="27">
+        <f>IF(S5="",1,S5^4/(C5^4+S5^4))</f>
+        <v/>
       </c>
     </row>
     <row r="6" ht="46" customHeight="1">
-      <c r="A6" s="27" t="n"/>
+      <c r="A6" s="28" t="n"/>
       <c r="B6" s="20" t="inlineStr">
         <is>
           <t>L03</t>
         </is>
       </c>
-      <c r="C6" s="21" t="n"/>
+      <c r="C6" s="21" t="n">
+        <v>4.15</v>
+      </c>
       <c r="D6" s="22" t="inlineStr">
         <is>
           <t>1/8</t>
         </is>
       </c>
       <c r="E6" s="23">
-        <f>Datos!$B$9*H6/100+VLOOKUP($A$4,Datos!$A$16:$C$17,2,0)+VLOOKUP($A$4,Datos!$A$16:$C$17,3,0)</f>
+        <f>(Datos!$B$9*H6/100+VLOOKUP($A$4,Datos!$A$16:$C$17,2,0)+VLOOKUP($A$4,Datos!$A$16:$C$17,3,0))*T6</f>
         <v/>
       </c>
       <c r="F6" s="7" t="n"/>
@@ -1627,27 +1719,30 @@
         <f>IF(C6="","",IF(VLOOKUP(D6,Datos!$A$21:$D$25,4,0)="Voladizo","---",P6))</f>
         <v/>
       </c>
-      <c r="R6" s="26" t="inlineStr">
-        <is>
-          <t>Falta la luz: completar en la columna LUZ y recalcula todo.</t>
-        </is>
+      <c r="R6" s="10" t="n"/>
+      <c r="S6" s="26" t="n"/>
+      <c r="T6" s="27">
+        <f>IF(S6="",1,S6^4/(C6^4+S6^4))</f>
+        <v/>
       </c>
     </row>
     <row r="7" ht="46" customHeight="1">
-      <c r="A7" s="27" t="n"/>
+      <c r="A7" s="28" t="n"/>
       <c r="B7" s="20" t="inlineStr">
         <is>
           <t>L04</t>
         </is>
       </c>
-      <c r="C7" s="21" t="n"/>
+      <c r="C7" s="21" t="n">
+        <v>3.73</v>
+      </c>
       <c r="D7" s="22" t="inlineStr">
         <is>
           <t>1/8</t>
         </is>
       </c>
       <c r="E7" s="23">
-        <f>Datos!$B$9*H7/100+VLOOKUP($A$4,Datos!$A$16:$C$17,2,0)+VLOOKUP($A$4,Datos!$A$16:$C$17,3,0)</f>
+        <f>(Datos!$B$9*H7/100+VLOOKUP($A$4,Datos!$A$16:$C$17,2,0)+VLOOKUP($A$4,Datos!$A$16:$C$17,3,0))*T7</f>
         <v/>
       </c>
       <c r="F7" s="7" t="n"/>
@@ -1692,27 +1787,30 @@
         <f>IF(C7="","",IF(VLOOKUP(D7,Datos!$A$21:$D$25,4,0)="Voladizo","---",P7))</f>
         <v/>
       </c>
-      <c r="R7" s="26" t="inlineStr">
-        <is>
-          <t>Falta la luz: completar en la columna LUZ y recalcula todo.</t>
-        </is>
+      <c r="R7" s="10" t="n"/>
+      <c r="S7" s="26" t="n"/>
+      <c r="T7" s="27">
+        <f>IF(S7="",1,S7^4/(C7^4+S7^4))</f>
+        <v/>
       </c>
     </row>
     <row r="8" ht="46" customHeight="1">
-      <c r="A8" s="27" t="n"/>
+      <c r="A8" s="28" t="n"/>
       <c r="B8" s="20" t="inlineStr">
         <is>
           <t>L05</t>
         </is>
       </c>
-      <c r="C8" s="21" t="n"/>
+      <c r="C8" s="21" t="n">
+        <v>3.73</v>
+      </c>
       <c r="D8" s="22" t="inlineStr">
         <is>
           <t>1/8</t>
         </is>
       </c>
       <c r="E8" s="23">
-        <f>Datos!$B$9*H8/100+VLOOKUP($A$4,Datos!$A$16:$C$17,2,0)+VLOOKUP($A$4,Datos!$A$16:$C$17,3,0)</f>
+        <f>(Datos!$B$9*H8/100+VLOOKUP($A$4,Datos!$A$16:$C$17,2,0)+VLOOKUP($A$4,Datos!$A$16:$C$17,3,0))*T8</f>
         <v/>
       </c>
       <c r="F8" s="7" t="n"/>
@@ -1757,27 +1855,30 @@
         <f>IF(C8="","",IF(VLOOKUP(D8,Datos!$A$21:$D$25,4,0)="Voladizo","---",P8))</f>
         <v/>
       </c>
-      <c r="R8" s="26" t="inlineStr">
-        <is>
-          <t>Falta la luz: completar en la columna LUZ y recalcula todo.</t>
-        </is>
+      <c r="R8" s="10" t="n"/>
+      <c r="S8" s="26" t="n"/>
+      <c r="T8" s="27">
+        <f>IF(S8="",1,S8^4/(C8^4+S8^4))</f>
+        <v/>
       </c>
     </row>
     <row r="9" ht="46" customHeight="1">
-      <c r="A9" s="27" t="n"/>
+      <c r="A9" s="28" t="n"/>
       <c r="B9" s="20" t="inlineStr">
         <is>
           <t>L06</t>
         </is>
       </c>
-      <c r="C9" s="21" t="n"/>
+      <c r="C9" s="21" t="n">
+        <v>2.15</v>
+      </c>
       <c r="D9" s="22" t="inlineStr">
         <is>
           <t>1/8</t>
         </is>
       </c>
       <c r="E9" s="23">
-        <f>Datos!$B$9*H9/100+VLOOKUP($A$4,Datos!$A$16:$C$17,2,0)+VLOOKUP($A$4,Datos!$A$16:$C$17,3,0)</f>
+        <f>(Datos!$B$9*H9/100+VLOOKUP($A$4,Datos!$A$16:$C$17,2,0)+VLOOKUP($A$4,Datos!$A$16:$C$17,3,0))*T9</f>
         <v/>
       </c>
       <c r="F9" s="7" t="n"/>
@@ -1822,27 +1923,30 @@
         <f>IF(C9="","",IF(VLOOKUP(D9,Datos!$A$21:$D$25,4,0)="Voladizo","---",P9))</f>
         <v/>
       </c>
-      <c r="R9" s="26" t="inlineStr">
-        <is>
-          <t>Falta la luz: completar en la columna LUZ y recalcula todo.</t>
-        </is>
+      <c r="R9" s="10" t="n"/>
+      <c r="S9" s="26" t="n"/>
+      <c r="T9" s="27">
+        <f>IF(S9="",1,S9^4/(C9^4+S9^4))</f>
+        <v/>
       </c>
     </row>
     <row r="10" ht="46" customHeight="1">
-      <c r="A10" s="27" t="n"/>
+      <c r="A10" s="28" t="n"/>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>L07</t>
-        </is>
-      </c>
-      <c r="C10" s="21" t="n"/>
+          <t>L07 (x)</t>
+        </is>
+      </c>
+      <c r="C10" s="21" t="n">
+        <v>4.85</v>
+      </c>
       <c r="D10" s="22" t="inlineStr">
         <is>
           <t>1/8</t>
         </is>
       </c>
       <c r="E10" s="23">
-        <f>Datos!$B$9*H10/100+VLOOKUP($A$4,Datos!$A$16:$C$17,2,0)+VLOOKUP($A$4,Datos!$A$16:$C$17,3,0)</f>
+        <f>(Datos!$B$9*H10/100+VLOOKUP($A$4,Datos!$A$16:$C$17,2,0)+VLOOKUP($A$4,Datos!$A$16:$C$17,3,0))*T10</f>
         <v/>
       </c>
       <c r="F10" s="7" t="n"/>
@@ -1887,233 +1991,408 @@
         <f>IF(C10="","",IF(VLOOKUP(D10,Datos!$A$21:$D$25,4,0)="Voladizo","---",P10))</f>
         <v/>
       </c>
-      <c r="R10" s="26" t="inlineStr">
-        <is>
-          <t>Falta la luz: completar en la columna LUZ y recalcula todo.</t>
-        </is>
+      <c r="R10" s="29" t="inlineStr">
+        <is>
+          <t>Losa cruzada 4,85 x 5,60 (ly/lx = 1,15). Direccion corta: toma el 64% de la carga por reparto de Marcus.</t>
+        </is>
+      </c>
+      <c r="S10" s="26" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="T10" s="27">
+        <f>IF(S10="",1,S10^4/(C10^4+S10^4))</f>
+        <v/>
       </c>
     </row>
     <row r="11" ht="46" customHeight="1">
       <c r="A11" s="28" t="n"/>
-      <c r="B11" s="29" t="inlineStr">
+      <c r="B11" s="20" t="inlineStr">
+        <is>
+          <t>L07 (y)</t>
+        </is>
+      </c>
+      <c r="C11" s="21" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="D11" s="22" t="inlineStr">
+        <is>
+          <t>1/8</t>
+        </is>
+      </c>
+      <c r="E11" s="23">
+        <f>(Datos!$B$9*H11/100+VLOOKUP($A$4,Datos!$A$16:$C$17,2,0)+VLOOKUP($A$4,Datos!$A$16:$C$17,3,0))*T11</f>
+        <v/>
+      </c>
+      <c r="F11" s="7" t="n"/>
+      <c r="G11" s="24">
+        <f>H11-Datos!$B$10</f>
+        <v/>
+      </c>
+      <c r="H11" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="I11" s="23">
+        <f>IF(C11="","",VLOOKUP(D11,Datos!$A$21:$D$25,2,0)*E11*C11^2)</f>
+        <v/>
+      </c>
+      <c r="J11" s="25">
+        <f>IF(I11="","",MAX(I11*100/(Datos!$B$7*Datos!$B$8*G11),Datos!$B$13))</f>
+        <v/>
+      </c>
+      <c r="K11" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="L11" s="7">
+        <f>IF(J11="","",MIN(Datos!$B$11,ROUND(100*PI()*(K11/10)^2/4/J11,0)))</f>
+        <v/>
+      </c>
+      <c r="M11" s="25">
+        <f>IF(J11="","",MAX(Datos!$B$12*J11,Datos!$B$13))</f>
+        <v/>
+      </c>
+      <c r="N11" s="22" t="n">
+        <v>6</v>
+      </c>
+      <c r="O11" s="7">
+        <f>IF(M11="","",MIN(Datos!$B$11,ROUND(100*PI()*(N11/10)^2/4/M11,0)))</f>
+        <v/>
+      </c>
+      <c r="P11" s="23">
+        <f>IF(C11="","",VLOOKUP(D11,Datos!$A$21:$D$25,3,0)*E11*C11)</f>
+        <v/>
+      </c>
+      <c r="Q11" s="23">
+        <f>IF(C11="","",IF(VLOOKUP(D11,Datos!$A$21:$D$25,4,0)="Voladizo","---",P11))</f>
+        <v/>
+      </c>
+      <c r="R11" s="29" t="inlineStr">
+        <is>
+          <t>Misma losa, direccion larga: toma el 36% restante. La armadura va cruzada con la fila anterior.</t>
+        </is>
+      </c>
+      <c r="S11" s="26" t="n">
+        <v>4.85</v>
+      </c>
+      <c r="T11" s="27">
+        <f>IF(S11="",1,S11^4/(C11^4+S11^4))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="46" customHeight="1">
+      <c r="A12" s="30" t="n"/>
+      <c r="B12" s="31" t="inlineStr">
         <is>
           <t>L08</t>
         </is>
       </c>
-      <c r="C11" s="30" t="n"/>
-      <c r="D11" s="31" t="inlineStr">
+      <c r="C12" s="32" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D12" s="33" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="E12" s="34">
+        <f>(Datos!$B$9*H12/100+VLOOKUP($A$4,Datos!$A$16:$C$17,2,0)+VLOOKUP($A$4,Datos!$A$16:$C$17,3,0))*T12</f>
+        <v/>
+      </c>
+      <c r="F12" s="35" t="n"/>
+      <c r="G12" s="36">
+        <f>H12-Datos!$B$10</f>
+        <v/>
+      </c>
+      <c r="H12" s="33" t="n">
+        <v>10</v>
+      </c>
+      <c r="I12" s="34">
+        <f>IF(C12="","",VLOOKUP(D12,Datos!$A$21:$D$25,2,0)*E12*C12^2)</f>
+        <v/>
+      </c>
+      <c r="J12" s="37">
+        <f>IF(I12="","",MAX(I12*100/(Datos!$B$7*Datos!$B$8*G12),Datos!$B$13))</f>
+        <v/>
+      </c>
+      <c r="K12" s="33" t="n">
+        <v>12</v>
+      </c>
+      <c r="L12" s="35">
+        <f>IF(J12="","",MIN(Datos!$B$11,ROUND(100*PI()*(K12/10)^2/4/J12,0)))</f>
+        <v/>
+      </c>
+      <c r="M12" s="37">
+        <f>IF(J12="","",MAX(Datos!$B$12*J12,Datos!$B$13))</f>
+        <v/>
+      </c>
+      <c r="N12" s="33" t="n">
+        <v>6</v>
+      </c>
+      <c r="O12" s="35">
+        <f>IF(M12="","",MIN(Datos!$B$11,ROUND(100*PI()*(N12/10)^2/4/M12,0)))</f>
+        <v/>
+      </c>
+      <c r="P12" s="34">
+        <f>IF(C12="","",VLOOKUP(D12,Datos!$A$21:$D$25,3,0)*E12*C12)</f>
+        <v/>
+      </c>
+      <c r="Q12" s="34">
+        <f>IF(C12="","",IF(VLOOKUP(D12,Datos!$A$21:$D$25,4,0)="Voladizo","---",P12))</f>
+        <v/>
+      </c>
+      <c r="R12" s="38" t="inlineStr">
+        <is>
+          <t>Voladizo: un solo apoyo.</t>
+        </is>
+      </c>
+      <c r="S12" s="39" t="n"/>
+      <c r="T12" s="40">
+        <f>IF(S12="",1,S12^4/(C12^4+S12^4))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="46" customHeight="1">
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>S/PA</t>
+        </is>
+      </c>
+      <c r="B13" s="20" t="inlineStr">
+        <is>
+          <t>L09</t>
+        </is>
+      </c>
+      <c r="C13" s="21" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="D13" s="22" t="inlineStr">
         <is>
           <t>1/8</t>
         </is>
       </c>
-      <c r="E11" s="32">
-        <f>Datos!$B$9*H11/100+VLOOKUP($A$4,Datos!$A$16:$C$17,2,0)+VLOOKUP($A$4,Datos!$A$16:$C$17,3,0)</f>
-        <v/>
-      </c>
-      <c r="F11" s="33" t="n"/>
-      <c r="G11" s="34">
-        <f>H11-Datos!$B$10</f>
-        <v/>
-      </c>
-      <c r="H11" s="31" t="n">
-        <v>10</v>
-      </c>
-      <c r="I11" s="32">
-        <f>IF(C11="","",VLOOKUP(D11,Datos!$A$21:$D$25,2,0)*E11*C11^2)</f>
-        <v/>
-      </c>
-      <c r="J11" s="35">
-        <f>IF(I11="","",MAX(I11*100/(Datos!$B$7*Datos!$B$8*G11),Datos!$B$13))</f>
-        <v/>
-      </c>
-      <c r="K11" s="31" t="n">
+      <c r="E13" s="23">
+        <f>(Datos!$B$9*H13/100+VLOOKUP($A$13,Datos!$A$16:$C$17,2,0)+VLOOKUP($A$13,Datos!$A$16:$C$17,3,0))*T13</f>
+        <v/>
+      </c>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="24">
+        <f>H13-Datos!$B$10</f>
+        <v/>
+      </c>
+      <c r="H13" s="22" t="n">
+        <v>13</v>
+      </c>
+      <c r="I13" s="23">
+        <f>IF(C13="","",VLOOKUP(D13,Datos!$A$21:$D$25,2,0)*E13*C13^2)</f>
+        <v/>
+      </c>
+      <c r="J13" s="25">
+        <f>IF(I13="","",MAX(I13*100/(Datos!$B$7*Datos!$B$8*G13),Datos!$B$13))</f>
+        <v/>
+      </c>
+      <c r="K13" s="22" t="n">
         <v>12</v>
       </c>
-      <c r="L11" s="33">
-        <f>IF(J11="","",MIN(Datos!$B$11,ROUND(100*PI()*(K11/10)^2/4/J11,0)))</f>
-        <v/>
-      </c>
-      <c r="M11" s="35">
-        <f>IF(J11="","",MAX(Datos!$B$12*J11,Datos!$B$13))</f>
-        <v/>
-      </c>
-      <c r="N11" s="31" t="n">
+      <c r="L13" s="7">
+        <f>IF(J13="","",MIN(Datos!$B$11,ROUND(100*PI()*(K13/10)^2/4/J13,0)))</f>
+        <v/>
+      </c>
+      <c r="M13" s="25">
+        <f>IF(J13="","",MAX(Datos!$B$12*J13,Datos!$B$13))</f>
+        <v/>
+      </c>
+      <c r="N13" s="22" t="n">
         <v>6</v>
       </c>
-      <c r="O11" s="33">
-        <f>IF(M11="","",MIN(Datos!$B$11,ROUND(100*PI()*(N11/10)^2/4/M11,0)))</f>
-        <v/>
-      </c>
-      <c r="P11" s="32">
-        <f>IF(C11="","",VLOOKUP(D11,Datos!$A$21:$D$25,3,0)*E11*C11)</f>
-        <v/>
-      </c>
-      <c r="Q11" s="32">
-        <f>IF(C11="","",IF(VLOOKUP(D11,Datos!$A$21:$D$25,4,0)="Voladizo","---",P11))</f>
-        <v/>
-      </c>
-      <c r="R11" s="36" t="inlineStr">
-        <is>
-          <t>Falta la luz: completar en la columna LUZ y recalcula todo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="46" customHeight="1">
-      <c r="A12" s="19" t="inlineStr">
-        <is>
-          <t>S/PA</t>
-        </is>
-      </c>
-      <c r="B12" s="20" t="inlineStr">
-        <is>
-          <t>L09</t>
-        </is>
-      </c>
-      <c r="C12" s="21" t="n"/>
-      <c r="D12" s="22" t="inlineStr">
+      <c r="O13" s="7">
+        <f>IF(M13="","",MIN(Datos!$B$11,ROUND(100*PI()*(N13/10)^2/4/M13,0)))</f>
+        <v/>
+      </c>
+      <c r="P13" s="23">
+        <f>IF(C13="","",VLOOKUP(D13,Datos!$A$21:$D$25,3,0)*E13*C13)</f>
+        <v/>
+      </c>
+      <c r="Q13" s="23">
+        <f>IF(C13="","",IF(VLOOKUP(D13,Datos!$A$21:$D$25,4,0)="Voladizo","---",P13))</f>
+        <v/>
+      </c>
+      <c r="R13" s="10" t="n"/>
+      <c r="S13" s="26" t="n"/>
+      <c r="T13" s="27">
+        <f>IF(S13="",1,S13^4/(C13^4+S13^4))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="46" customHeight="1">
+      <c r="A14" s="28" t="n"/>
+      <c r="B14" s="20" t="inlineStr">
+        <is>
+          <t>L10 (x)</t>
+        </is>
+      </c>
+      <c r="C14" s="21" t="n">
+        <v>4.85</v>
+      </c>
+      <c r="D14" s="22" t="inlineStr">
         <is>
           <t>1/8</t>
         </is>
       </c>
-      <c r="E12" s="23">
-        <f>Datos!$B$9*H12/100+VLOOKUP($A$12,Datos!$A$16:$C$17,2,0)+VLOOKUP($A$12,Datos!$A$16:$C$17,3,0)</f>
-        <v/>
-      </c>
-      <c r="F12" s="7" t="n"/>
-      <c r="G12" s="24">
-        <f>H12-Datos!$B$10</f>
-        <v/>
-      </c>
-      <c r="H12" s="22" t="n">
-        <v>13</v>
-      </c>
-      <c r="I12" s="23">
-        <f>IF(C12="","",VLOOKUP(D12,Datos!$A$21:$D$25,2,0)*E12*C12^2)</f>
-        <v/>
-      </c>
-      <c r="J12" s="25">
-        <f>IF(I12="","",MAX(I12*100/(Datos!$B$7*Datos!$B$8*G12),Datos!$B$13))</f>
-        <v/>
-      </c>
-      <c r="K12" s="22" t="n">
+      <c r="E14" s="23">
+        <f>(Datos!$B$9*H14/100+VLOOKUP($A$13,Datos!$A$16:$C$17,2,0)+VLOOKUP($A$13,Datos!$A$16:$C$17,3,0))*T14</f>
+        <v/>
+      </c>
+      <c r="F14" s="7" t="n"/>
+      <c r="G14" s="24">
+        <f>H14-Datos!$B$10</f>
+        <v/>
+      </c>
+      <c r="H14" s="22" t="n">
         <v>12</v>
       </c>
-      <c r="L12" s="7">
-        <f>IF(J12="","",MIN(Datos!$B$11,ROUND(100*PI()*(K12/10)^2/4/J12,0)))</f>
-        <v/>
-      </c>
-      <c r="M12" s="25">
-        <f>IF(J12="","",MAX(Datos!$B$12*J12,Datos!$B$13))</f>
-        <v/>
-      </c>
-      <c r="N12" s="22" t="n">
+      <c r="I14" s="23">
+        <f>IF(C14="","",VLOOKUP(D14,Datos!$A$21:$D$25,2,0)*E14*C14^2)</f>
+        <v/>
+      </c>
+      <c r="J14" s="25">
+        <f>IF(I14="","",MAX(I14*100/(Datos!$B$7*Datos!$B$8*G14),Datos!$B$13))</f>
+        <v/>
+      </c>
+      <c r="K14" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="L14" s="7">
+        <f>IF(J14="","",MIN(Datos!$B$11,ROUND(100*PI()*(K14/10)^2/4/J14,0)))</f>
+        <v/>
+      </c>
+      <c r="M14" s="25">
+        <f>IF(J14="","",MAX(Datos!$B$12*J14,Datos!$B$13))</f>
+        <v/>
+      </c>
+      <c r="N14" s="22" t="n">
         <v>6</v>
       </c>
-      <c r="O12" s="7">
-        <f>IF(M12="","",MIN(Datos!$B$11,ROUND(100*PI()*(N12/10)^2/4/M12,0)))</f>
-        <v/>
-      </c>
-      <c r="P12" s="23">
-        <f>IF(C12="","",VLOOKUP(D12,Datos!$A$21:$D$25,3,0)*E12*C12)</f>
-        <v/>
-      </c>
-      <c r="Q12" s="23">
-        <f>IF(C12="","",IF(VLOOKUP(D12,Datos!$A$21:$D$25,4,0)="Voladizo","---",P12))</f>
-        <v/>
-      </c>
-      <c r="R12" s="26" t="inlineStr">
-        <is>
-          <t>Falta la luz: completar en la columna LUZ y recalcula todo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="46" customHeight="1">
-      <c r="A13" s="28" t="n"/>
-      <c r="B13" s="29" t="inlineStr">
-        <is>
-          <t>L10</t>
-        </is>
-      </c>
-      <c r="C13" s="30" t="n"/>
-      <c r="D13" s="31" t="inlineStr">
+      <c r="O14" s="7">
+        <f>IF(M14="","",MIN(Datos!$B$11,ROUND(100*PI()*(N14/10)^2/4/M14,0)))</f>
+        <v/>
+      </c>
+      <c r="P14" s="23">
+        <f>IF(C14="","",VLOOKUP(D14,Datos!$A$21:$D$25,3,0)*E14*C14)</f>
+        <v/>
+      </c>
+      <c r="Q14" s="23">
+        <f>IF(C14="","",IF(VLOOKUP(D14,Datos!$A$21:$D$25,4,0)="Voladizo","---",P14))</f>
+        <v/>
+      </c>
+      <c r="R14" s="29" t="inlineStr">
+        <is>
+          <t>Losa cruzada 4,85 x 6,00 (ly/lx = 1,24). Direccion corta: toma el 70% de la carga por reparto de Marcus.</t>
+        </is>
+      </c>
+      <c r="S14" s="26" t="n">
+        <v>6</v>
+      </c>
+      <c r="T14" s="27">
+        <f>IF(S14="",1,S14^4/(C14^4+S14^4))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="46" customHeight="1">
+      <c r="A15" s="30" t="n"/>
+      <c r="B15" s="31" t="inlineStr">
+        <is>
+          <t>L10 (y)</t>
+        </is>
+      </c>
+      <c r="C15" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="D15" s="33" t="inlineStr">
         <is>
           <t>1/8</t>
         </is>
       </c>
-      <c r="E13" s="32">
-        <f>Datos!$B$9*H13/100+VLOOKUP($A$12,Datos!$A$16:$C$17,2,0)+VLOOKUP($A$12,Datos!$A$16:$C$17,3,0)</f>
-        <v/>
-      </c>
-      <c r="F13" s="33" t="n"/>
-      <c r="G13" s="34">
-        <f>H13-Datos!$B$10</f>
-        <v/>
-      </c>
-      <c r="H13" s="31" t="n">
+      <c r="E15" s="34">
+        <f>(Datos!$B$9*H15/100+VLOOKUP($A$13,Datos!$A$16:$C$17,2,0)+VLOOKUP($A$13,Datos!$A$16:$C$17,3,0))*T15</f>
+        <v/>
+      </c>
+      <c r="F15" s="35" t="n"/>
+      <c r="G15" s="36">
+        <f>H15-Datos!$B$10</f>
+        <v/>
+      </c>
+      <c r="H15" s="33" t="n">
         <v>12</v>
       </c>
-      <c r="I13" s="32">
-        <f>IF(C13="","",VLOOKUP(D13,Datos!$A$21:$D$25,2,0)*E13*C13^2)</f>
-        <v/>
-      </c>
-      <c r="J13" s="35">
-        <f>IF(I13="","",MAX(I13*100/(Datos!$B$7*Datos!$B$8*G13),Datos!$B$13))</f>
-        <v/>
-      </c>
-      <c r="K13" s="31" t="n">
+      <c r="I15" s="34">
+        <f>IF(C15="","",VLOOKUP(D15,Datos!$A$21:$D$25,2,0)*E15*C15^2)</f>
+        <v/>
+      </c>
+      <c r="J15" s="37">
+        <f>IF(I15="","",MAX(I15*100/(Datos!$B$7*Datos!$B$8*G15),Datos!$B$13))</f>
+        <v/>
+      </c>
+      <c r="K15" s="33" t="n">
         <v>12</v>
       </c>
-      <c r="L13" s="33">
-        <f>IF(J13="","",MIN(Datos!$B$11,ROUND(100*PI()*(K13/10)^2/4/J13,0)))</f>
-        <v/>
-      </c>
-      <c r="M13" s="35">
-        <f>IF(J13="","",MAX(Datos!$B$12*J13,Datos!$B$13))</f>
-        <v/>
-      </c>
-      <c r="N13" s="31" t="n">
+      <c r="L15" s="35">
+        <f>IF(J15="","",MIN(Datos!$B$11,ROUND(100*PI()*(K15/10)^2/4/J15,0)))</f>
+        <v/>
+      </c>
+      <c r="M15" s="37">
+        <f>IF(J15="","",MAX(Datos!$B$12*J15,Datos!$B$13))</f>
+        <v/>
+      </c>
+      <c r="N15" s="33" t="n">
         <v>6</v>
       </c>
-      <c r="O13" s="33">
-        <f>IF(M13="","",MIN(Datos!$B$11,ROUND(100*PI()*(N13/10)^2/4/M13,0)))</f>
-        <v/>
-      </c>
-      <c r="P13" s="32">
-        <f>IF(C13="","",VLOOKUP(D13,Datos!$A$21:$D$25,3,0)*E13*C13)</f>
-        <v/>
-      </c>
-      <c r="Q13" s="32">
-        <f>IF(C13="","",IF(VLOOKUP(D13,Datos!$A$21:$D$25,4,0)="Voladizo","---",P13))</f>
-        <v/>
-      </c>
-      <c r="R13" s="36" t="inlineStr">
-        <is>
-          <t>Falta la luz: completar en la columna LUZ y recalcula todo.</t>
-        </is>
+      <c r="O15" s="35">
+        <f>IF(M15="","",MIN(Datos!$B$11,ROUND(100*PI()*(N15/10)^2/4/M15,0)))</f>
+        <v/>
+      </c>
+      <c r="P15" s="34">
+        <f>IF(C15="","",VLOOKUP(D15,Datos!$A$21:$D$25,3,0)*E15*C15)</f>
+        <v/>
+      </c>
+      <c r="Q15" s="34">
+        <f>IF(C15="","",IF(VLOOKUP(D15,Datos!$A$21:$D$25,4,0)="Voladizo","---",P15))</f>
+        <v/>
+      </c>
+      <c r="R15" s="38" t="inlineStr">
+        <is>
+          <t>Misma losa, direccion larga: toma el 30% restante. La armadura va cruzada con la fila anterior.</t>
+        </is>
+      </c>
+      <c r="S15" s="39" t="n">
+        <v>4.85</v>
+      </c>
+      <c r="T15" s="40">
+        <f>IF(S15="",1,S15^4/(C15^4+S15^4))</f>
+        <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="15">
+    <mergeCell ref="A1:T1"/>
     <mergeCell ref="J2:L2"/>
-    <mergeCell ref="A4:A11"/>
+    <mergeCell ref="S2:T2"/>
     <mergeCell ref="G2:H2"/>
+    <mergeCell ref="C2:C3"/>
     <mergeCell ref="E2:F2"/>
-    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="A4:A12"/>
     <mergeCell ref="P2:Q2"/>
-    <mergeCell ref="D2:D3"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="A2:A3"/>
-    <mergeCell ref="A1:R1"/>
-    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
     <mergeCell ref="R2:R3"/>
     <mergeCell ref="M2:O2"/>
     <mergeCell ref="I2:I3"/>
+    <mergeCell ref="A13:A15"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="D4:D13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D4:D15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Datos!$A$21:$A$25</formula1>
     </dataValidation>
-    <dataValidation sqref="K4:K13 N4:N13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K4:K15 N4:N15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"6,8,10,12,16"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2129,7 +2408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B35"/>
+  <dimension ref="A1:B44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2137,296 +2416,368 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="37" t="inlineStr">
+      <c r="A1" s="41" t="inlineStr">
         <is>
           <t>MEMORIA DE CALCULO - LOSAS</t>
         </is>
       </c>
-      <c r="B1" s="38" t="inlineStr"/>
+      <c r="B1" s="42" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="38" t="inlineStr"/>
-      <c r="B2" s="39" t="inlineStr"/>
+      <c r="A2" s="42" t="inlineStr"/>
+      <c r="B2" s="43" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="38" t="inlineStr">
+      <c r="A3" s="42" t="inlineStr">
         <is>
           <t>METODO</t>
         </is>
       </c>
-      <c r="B3" s="38" t="inlineStr">
+      <c r="B3" s="42" t="inlineStr">
         <is>
           <t>Tensiones admisibles, igual criterio que la planilla modelo de la catedra.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="38" t="inlineStr"/>
-      <c r="B4" s="39" t="inlineStr">
+      <c r="A4" s="42" t="inlineStr"/>
+      <c r="B4" s="43" t="inlineStr">
         <is>
           <t>Se verifico contra la fila de ejemplo: momentos y reacciones coinciden exactamente.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="38" t="inlineStr">
+      <c r="A5" s="42" t="inlineStr">
         <is>
           <t>MATERIALES</t>
         </is>
       </c>
-      <c r="B5" s="38" t="inlineStr">
+      <c r="B5" s="42" t="inlineStr">
         <is>
           <t>H-21 (f'c 210 kg/cm2). Acero 42/50 (fy 4200). Tension admisible 2400 kg/cm2.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="38" t="inlineStr">
+      <c r="A6" s="42" t="inlineStr">
         <is>
           <t>DIMENSIONES</t>
         </is>
       </c>
-      <c r="B6" s="38" t="inlineStr">
+      <c r="B6" s="42" t="inlineStr">
         <is>
           <t>h = altura util | d = espesor total. Recubrimiento 1,5 cm.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="38" t="inlineStr"/>
-      <c r="B7" s="39" t="inlineStr"/>
+      <c r="A7" s="42" t="inlineStr"/>
+      <c r="B7" s="43" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="38" t="inlineStr">
+      <c r="A8" s="42" t="inlineStr">
         <is>
           <t>1. CARGAS</t>
         </is>
       </c>
-      <c r="B8" s="38" t="inlineStr">
+      <c r="B8" s="42" t="inlineStr">
         <is>
           <t>p = peso propio + terminaciones + q      (cargas de servicio, sin mayorar)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="38" t="inlineStr"/>
-      <c r="B9" s="39" t="inlineStr">
+      <c r="A9" s="42" t="inlineStr"/>
+      <c r="B9" s="43" t="inlineStr">
         <is>
           <t>Peso propio = 2400 x d / 100, calculado con el espesor propio de cada losa.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="38" t="inlineStr">
+      <c r="A10" s="42" t="inlineStr">
         <is>
           <t>S/PB</t>
         </is>
       </c>
-      <c r="B10" s="39" t="inlineStr">
+      <c r="B10" s="43" t="inlineStr">
         <is>
           <t>Terminaciones 242 kg/m2 (contrapiso 130 + carpeta 42 + piso 50 + cielorraso 20)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="38" t="inlineStr"/>
-      <c r="B11" s="39" t="inlineStr">
+      <c r="A11" s="42" t="inlineStr"/>
+      <c r="B11" s="43" t="inlineStr">
         <is>
           <t>q = 200 kg/m2 (vivienda)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="38" t="inlineStr">
+      <c r="A12" s="42" t="inlineStr">
         <is>
           <t>S/PA</t>
         </is>
       </c>
-      <c r="B12" s="39" t="inlineStr">
+      <c r="B12" s="43" t="inlineStr">
         <is>
           <t>Terminaciones 252 kg/m2 (contrapiso pendiente 140 + carpeta 42 + aislacion 50 +</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="38" t="inlineStr"/>
-      <c r="B13" s="39" t="inlineStr">
+      <c r="A13" s="42" t="inlineStr"/>
+      <c r="B13" s="43" t="inlineStr">
         <is>
           <t>cielorraso 20).  q = 100 kg/m2 (azotea no accesible)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="38" t="inlineStr"/>
-      <c r="B14" s="39" t="inlineStr"/>
+      <c r="A14" s="42" t="inlineStr"/>
+      <c r="B14" s="43" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="38" t="inlineStr">
+      <c r="A15" s="42" t="inlineStr">
         <is>
           <t>2. SOLICITACIONES</t>
         </is>
       </c>
-      <c r="B15" s="38" t="inlineStr">
+      <c r="B15" s="42" t="inlineStr">
         <is>
           <t>M = coeficiente x p x L2, segun el grado de empotramiento:</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="38" t="inlineStr"/>
-      <c r="B16" s="39" t="inlineStr">
+      <c r="A16" s="42" t="inlineStr"/>
+      <c r="B16" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">  1/8 simplemente apoyada    1/10 y 1/14 continua    1/12 biempotrada    1/2 voladizo</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="38" t="inlineStr"/>
-      <c r="B17" s="39" t="inlineStr">
+      <c r="A17" s="42" t="inlineStr"/>
+      <c r="B17" s="43" t="inlineStr">
         <is>
           <t>R = coeficiente x p x L. En voladizo Rx = p x L y Ry no corresponde.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="38" t="inlineStr"/>
-      <c r="B18" s="39" t="inlineStr"/>
+      <c r="A18" s="42" t="inlineStr"/>
+      <c r="B18" s="43" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="38" t="inlineStr">
+      <c r="A19" s="42" t="inlineStr">
         <is>
           <t>3. ARMADURA</t>
         </is>
       </c>
-      <c r="B19" s="38" t="inlineStr">
+      <c r="B19" s="42" t="inlineStr">
         <is>
           <t>As = M x 100 / (2400 x 0,9 x h)        [cm2/m]</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="38" t="inlineStr"/>
-      <c r="B20" s="39" t="inlineStr">
+      <c r="A20" s="42" t="inlineStr"/>
+      <c r="B20" s="43" t="inlineStr">
         <is>
           <t>separacion = 100 x area de la barra / As, redondeada, con maximo 20 cm</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="38" t="inlineStr"/>
-      <c r="B21" s="39" t="inlineStr">
+      <c r="A21" s="42" t="inlineStr"/>
+      <c r="B21" s="43" t="inlineStr">
         <is>
           <t>Armadura de reparticion = As / 5, con un minimo de 0,30 cm2/m</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="38" t="inlineStr"/>
-      <c r="B22" s="39" t="inlineStr"/>
+      <c r="A22" s="42" t="inlineStr"/>
+      <c r="B22" s="43" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="38" t="inlineStr">
+      <c r="A23" s="42" t="inlineStr">
         <is>
           <t>4. ESPESORES</t>
         </is>
       </c>
-      <c r="B23" s="38" t="inlineStr">
+      <c r="B23" s="42" t="inlineStr">
         <is>
           <t>Los espesores d se leyeron del plano: estan escritos debajo del rotulo de cada losa.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="38" t="inlineStr"/>
-      <c r="B24" s="39" t="inlineStr">
+      <c r="A24" s="42" t="inlineStr"/>
+      <c r="B24" s="43" t="inlineStr">
         <is>
           <t>S/PB:  L01 11 | L02 9 | L03 13 | L04 11 | L05 11 | L06 8 | L07 12 | L08 10</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="38" t="inlineStr"/>
-      <c r="B25" s="39" t="inlineStr">
+      <c r="A25" s="42" t="inlineStr"/>
+      <c r="B25" s="43" t="inlineStr">
         <is>
           <t>S/PA:  L09 13 | L10 12</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="38" t="inlineStr"/>
-      <c r="B26" s="39" t="inlineStr"/>
+      <c r="A26" s="42" t="inlineStr"/>
+      <c r="B26" s="43" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="38" t="inlineStr">
-        <is>
-          <t>5. FALTA LA LUZ</t>
-        </is>
-      </c>
-      <c r="B27" s="38" t="inlineStr">
-        <is>
-          <t>Es el unico dato que no se pudo obtener del plano. Las cruces dibujadas sobre</t>
+      <c r="A27" s="42" t="inlineStr">
+        <is>
+          <t>5. LUCES</t>
+        </is>
+      </c>
+      <c r="B27" s="42" t="inlineStr">
+        <is>
+          <t>Relevadas en obra y aportadas por el proyectista. Dos losas son voladizo</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="38" t="inlineStr"/>
-      <c r="B28" s="39" t="inlineStr">
-        <is>
-          <t>la planta marcan vacios, no losas, y los rotulos no traen la luz acotada.</t>
+      <c r="A28" s="42" t="inlineStr"/>
+      <c r="B28" s="43" t="inlineStr">
+        <is>
+          <t>(L02 de 0,80 m y L08 de 0,75 m) y se calculan con M = p L2 / 2.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="38" t="inlineStr"/>
-      <c r="B29" s="39" t="inlineStr">
-        <is>
-          <t>Completar la columna LUZ (naranja) de cada losa: el resto se calcula solo.</t>
-        </is>
-      </c>
+      <c r="A29" s="42" t="inlineStr"/>
+      <c r="B29" s="43" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="38" t="inlineStr"/>
-      <c r="B30" s="39" t="inlineStr">
-        <is>
-          <t>Ojo: la luz es la del sentido en que arma la losa, normalmente la luz corta.</t>
+      <c r="A30" s="42" t="inlineStr">
+        <is>
+          <t>6. LOSAS CRUZADAS</t>
+        </is>
+      </c>
+      <c r="B30" s="43" t="inlineStr">
+        <is>
+          <t>L07 (4,85 x 5,60) y L10 (4,85 x 6,00) apoyan en los cuatro bordes y su relacion</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="38" t="inlineStr"/>
-      <c r="B31" s="39" t="inlineStr"/>
+      <c r="A31" s="42" t="inlineStr"/>
+      <c r="B31" s="43" t="inlineStr">
+        <is>
+          <t>de lados es menor que 2, por lo que trabajan en las dos direcciones.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="38" t="inlineStr">
+      <c r="A32" s="42" t="inlineStr"/>
+      <c r="B32" s="43" t="inlineStr">
+        <is>
+          <t>Se reparte la carga por el metodo de Marcus:   kx = ly4 / (lx4 + ly4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="42" t="inlineStr"/>
+      <c r="B33" s="43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  L07: ly/lx = 1,15  -&gt;  64% en la direccion corta, 36% en la larga</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="42" t="inlineStr"/>
+      <c r="B34" s="43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  L10: ly/lx = 1,24  -&gt;  70% en la direccion corta, 30% en la larga</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="42" t="inlineStr"/>
+      <c r="B35" s="43" t="inlineStr">
+        <is>
+          <t>Cada una ocupa dos renglones, uno por direccion, con la fraccion de carga que</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="42" t="inlineStr"/>
+      <c r="B36" s="43" t="inlineStr">
+        <is>
+          <t>le toca ya aplicada en la columna CARGAS. Las dos armaduras se cruzan en obra:</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="42" t="inlineStr"/>
+      <c r="B37" s="43" t="inlineStr">
+        <is>
+          <t>la de la direccion corta va abajo, la de la larga arriba de aquella.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="42" t="inlineStr"/>
+      <c r="B38" s="43" t="inlineStr">
+        <is>
+          <t>La columna auxiliar luz transv. es la que dispara el reparto: si se borra, la</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="42" t="inlineStr"/>
+      <c r="B39" s="43" t="inlineStr">
+        <is>
+          <t>fila vuelve a calcularse como losa armada en una direccion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="42" t="inlineStr"/>
+      <c r="B40" s="43" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="42" t="inlineStr">
         <is>
           <t>LIMITACIONES</t>
         </is>
       </c>
-      <c r="B32" s="38" t="inlineStr">
-        <is>
-          <t>El grado de empotramiento viene precargado en 1/8 para todas. Corregirlo losa</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="38" t="inlineStr"/>
-      <c r="B33" s="39" t="inlineStr">
-        <is>
-          <t>por losa segun las condiciones de borde reales (continuidad sobre vigas, voladizos).</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="38" t="inlineStr"/>
-      <c r="B34" s="39" t="inlineStr">
+      <c r="B41" s="42" t="inlineStr">
+        <is>
+          <t>El grado de empotramiento esta cargado en 1/8 salvo los dos voladizos (1/2). Si</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="42" t="inlineStr"/>
+      <c r="B42" s="43" t="inlineStr">
+        <is>
+          <t>alguna losa es continua sobre una viga corresponde 1/10 o 1/14: corregir en la columna.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="42" t="inlineStr"/>
+      <c r="B43" s="43" t="inlineStr">
         <is>
           <t>El diagrama de cargas es una imagen fija: si cambias el grado, cambialo a mano.</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="38" t="inlineStr"/>
-      <c r="B35" s="39" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="42" t="inlineStr"/>
+      <c r="B44" s="43" t="inlineStr">
         <is>
           <t>Trabajo academico. Requiere verificacion y firma de profesional matriculado.</t>
         </is>

</xml_diff>